<commit_message>
v5.1.0: Wandeldarlehen-Testakte komplett ueberarbeitet
- Vollwertige bilinguale DE/EN Wandeldarlehen-Vertragsfassung (11 Paragraphen, Mustervorlage)
- Einsprachige deutsche Vertragsfassung passend dazu
- Neues Term-Sheet (24 Parameter, 15. April 2026) als Vor-Vertragsphase
- Neue Wandlungsmitteilung der Gesellschaft an den Investor
- Wandlungserklaerung, Gesellschafterbeschluss, Notar-Paket aufpoliert
- Cap-Tables Pre-/Post-Money sauber neu geschrieben (1.000 Anteile, ohne Treasury, mit Verwaesserungs-Check)
- MD-Konvertierung mit Bilingual-Pattern fuer lesbare GitHub-Vorschauen
- XLSX-Vorschauen mit Prozent-Format, Tausender-Trenner, Title-Bloecken
- 275 .md-Vorschauen im gesamten Repo neu generiert
- Testakten- und Plugin-Readme aktualisiert
</commit_message>
<xml_diff>
--- a/testakten/wandeldarlehen-beispielcase/Cap-Table-Pre-Money.xlsx
+++ b/testakten/wandeldarlehen-beispielcase/Cap-Table-Pre-Money.xlsx
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;EUR&quot;"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="7">
     <font>
       <name val="Calibri"/>
@@ -28,41 +26,34 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001B474D"/>
-      <sz val="14"/>
+      <color rgb="001F4E79"/>
+      <sz val="16"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <color rgb="007A7974"/>
-      <sz val="11"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <color rgb="0028251D"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="007A7974"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="0020808D"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -71,18 +62,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B474D"/>
-        <bgColor rgb="001B474D"/>
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0020808D"/>
-        <bgColor rgb="0020808D"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -92,62 +89,114 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D4D1CA"/>
+        <color rgb="00808080"/>
       </left>
       <right style="thin">
-        <color rgb="00D4D1CA"/>
+        <color rgb="00808080"/>
       </right>
       <top style="thin">
-        <color rgb="00D4D1CA"/>
+        <color rgb="00808080"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D4D1CA"/>
+        <color rgb="00808080"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -514,155 +563,369 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E13"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="6" customHeight="1"/>
-    <row r="2" ht="24" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Sonnenglas Solartechnologie UG (haftungsbeschränkt)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Cap-Table — Pre-Money (vor Wandlung / vor Seed-Runde)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="6" customHeight="1"/>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Gesellschafter</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Anteile (Stk.)</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Nennwert (EUR)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Beteiligung (%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Dr. Mira Schoeneck (GF)</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="D6" s="6">
-        <f>C6*1</f>
-        <v/>
-      </c>
-      <c r="E6" s="7">
-        <f>C6/C9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cap-Table Pre-Money — Sonnenglas Solartechnologie UG (haftungsbeschraenkt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Stand vor Auszahlung Wandeldarlehen Northstar Pre-Seed Partners GmbH &amp; Co. KG · Stichtag 15. April 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Eckdaten Gesellschaft</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Firma</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Sonnenglas Solartechnologie UG (haftungsbeschraenkt)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Sitz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Handelsregister</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>AG Charlottenburg HRB 123456 B</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Stammkapital</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>EUR 1.000,00</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Anzahl Geschaeftsanteile</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>1.000 Stueck zu je EUR 1,00 Nennbetrag</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Stichtag</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>15. April 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="7" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Gesellschafterstruktur</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Gesellschafter:in</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Adresse</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Geschaeftsanteile (Nrn.)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Anzahl</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Nennbetrag (EUR)</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Anteil am Stammkapital</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Dr. Mira Schoeneck</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Friedrichstrasse 88, 10117 Berlin</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>1 - 600</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>600</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Lina Habersaat</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>35</v>
-      </c>
-      <c r="D7" s="6">
-        <f>C7*1</f>
-        <v/>
-      </c>
-      <c r="E7" s="7">
-        <f>C7/C9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Sonnenglas UG (Treasury)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="D8" s="6">
-        <f>C8*1</f>
-        <v/>
-      </c>
-      <c r="E8" s="7">
-        <f>C8/C9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Gesamt</t>
-        </is>
-      </c>
-      <c r="C9" s="9">
-        <f>SUM(C6:C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="10">
-        <f>SUM(D6:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="11">
-        <f>SUM(E6:E8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Stammkapital: EUR 1.000,00 | 100 Anteile à EUR 1,00 | HRB 123456 B, AG Charlottenburg</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>Stand: vor Wandlung des Wandeldarlehens Northstar / vor Seed-Finanzierungsrunde</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>Wandeldarlehen Northstar Pre-Seed Partners: EUR 250.000 (ausstehend, noch nicht gewandelt)</t>
-        </is>
-      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Beispielweg 5, 22085 Hamburg</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>601 - 1000</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr"/>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>1 - 1000</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E16" s="16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Pro-forma Wandelannahmen (zur Information, noch nicht ausgeuebt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Wandeldarlehen Northstar</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Nominal EUR 250.000 + 6,0 % p.a. (act/360) bei voller Laufzeit</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Cap (Pre-Money)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>EUR 4.000.000</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>20 % auf Seed-Preis pro Anteil</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Erwartete Wandlungssumme (Cap-Szenario)</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>EUR 250.000,00 + EUR 11.541,67 Zinsen = EUR 261.541,67</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Cap-Preis je Geschaeftsanteil</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>EUR 4.000.000 / 1.000 = EUR 4.000,00</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Daraus rechnerisch neue Anteile bei Wandlung</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>65,3854 -&gt; kaufmaennisch aufgerundet 66 Anteile</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B2:E2"/>
+  <mergeCells count="17">
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B9:F9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>